<commit_message>
Move template version to ConceptScheme sheet
</commit_message>
<xml_diff>
--- a/src/voc4cat/templates/vocab/blank_043.xlsx
+++ b/src/voc4cat/templates/vocab/blank_043.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\MyProg\gh-nfdi4cat\voc4cat\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dlinke\MyProg_local\gh-nfdi4cat\voc4cat-tool\src\voc4cat\templates\vocab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CCFAF9A-16AB-4F1A-9E10-106FA17068AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1209A9-5678-4E59-91D2-38A6DB0E7FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="75" yWindow="8700" windowWidth="28500" windowHeight="8535" tabRatio="652" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9495" yWindow="5475" windowWidth="28800" windowHeight="15825" tabRatio="652" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="1" r:id="rId1"/>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="90">
   <si>
     <t>Template version</t>
   </si>
@@ -1474,6 +1474,15 @@
       </rPr>
       <t xml:space="preserve"> = A catalogue PID or DOI, e.g. eCat ID, if the vocab has one.</t>
     </r>
+  </si>
+  <si>
+    <t>Template Version</t>
+  </si>
+  <si>
+    <t>Version of the xlsx template</t>
+  </si>
+  <si>
+    <t>0.4.3, rev. 2025-07a</t>
   </si>
 </sst>
 </file>
@@ -5348,7 +5357,20 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
     <row r="14" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>